<commit_message>
Fix map color for homepage
</commit_message>
<xml_diff>
--- a/data/cesvi-indiceinfanzia_news.xlsx
+++ b/data/cesvi-indiceinfanzia_news.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>#</t>
   </si>
@@ -75,6 +75,15 @@
   <si>
     <t>https://cesvi.org/notizie/cesvi-presenta-a-roma-la-settima-edizione-dellindice-regionale-sul-maltrattamento-e-la-cura-allinfanzia-in-italia/?_gl=1*e5jsh5*_up*MQ..*_ga*MTc5NjAzMjIwMy4xNzgxMDIxMTU3*_ga_HCXHRSXJ9N*czE3ODEwMjExNTYkbzEkZzAkdDE3ODEwMjExNTYkajYwJGwwJGgw*_ga_BC2WH7M4X0*czE3ODEwMjExNTYkbzEkZzAkdDE3ODEwMjExNTYkajYwJGwwJGgw</t>
   </si>
+  <si>
+    <t>Infanzia, Cesvi: solitudine e povertà relazionale alimentano il maltrattamento</t>
+  </si>
+  <si>
+    <t>Il Sole 24 ORE</t>
+  </si>
+  <si>
+    <t>https://www.ilsole24ore.com/art/infanzia-cesvi-solitudine-e-poverta-relazionale-alimentano-maltrattamento-AIws6HaD?refresh_ce=1</t>
+  </si>
 </sst>
 </file>
 
@@ -83,7 +92,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12.0"/>
       <color theme="1"/>
@@ -93,17 +102,21 @@
     <font>
       <b/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Roboto Mono"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Roboto Mono"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Roboto Mono"/>
     </font>
     <font>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
-      <name val="Roboto"/>
     </font>
   </fonts>
   <fills count="2">
@@ -120,12 +133,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -142,7 +158,7 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -159,8 +175,8 @@
       <font/>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF356854"/>
-          <bgColor rgb="FF356854"/>
+          <fgColor rgb="FFEB6608"/>
+          <bgColor rgb="FFEB6608"/>
         </patternFill>
       </fill>
       <border/>
@@ -188,16 +204,16 @@
     <dxf>
       <border>
         <left style="thin">
-          <color rgb="FF356854"/>
+          <color rgb="FFEB6608"/>
         </left>
         <right style="thin">
-          <color rgb="FF356854"/>
+          <color rgb="FFEB6608"/>
         </right>
         <top style="thin">
-          <color rgb="FF356854"/>
+          <color rgb="FFEB6608"/>
         </top>
         <bottom style="thin">
-          <color rgb="FF356854"/>
+          <color rgb="FFEB6608"/>
         </bottom>
       </border>
     </dxf>
@@ -431,11 +447,12 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.78"/>
-    <col customWidth="1" min="2" max="2" width="11.44"/>
-    <col customWidth="1" min="3" max="3" width="89.78"/>
-    <col customWidth="1" min="4" max="4" width="10.67"/>
-    <col customWidth="1" min="5" max="27" width="8.33"/>
+    <col customWidth="1" min="1" max="1" width="8.89"/>
+    <col customWidth="1" min="2" max="2" width="12.67"/>
+    <col customWidth="1" min="3" max="3" width="124.67"/>
+    <col customWidth="1" min="4" max="4" width="11.33"/>
+    <col customWidth="1" min="5" max="5" width="24.78"/>
+    <col customWidth="1" min="6" max="27" width="8.33"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -451,233 +468,299 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>1.0</v>
       </c>
-      <c r="B2" s="3">
-        <v>46181.0</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="4">
+        <v>46183.0</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>2.0</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="E3" s="6"/>
+      <c r="B3" s="4">
+        <v>46183.0</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>3.0</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="E4" s="6"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="2">
+      <c r="A5" s="3">
         <v>4.0</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="E5" s="6"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="2">
+      <c r="A6" s="3">
         <v>5.0</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="E6" s="6"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="2">
+      <c r="A7" s="3">
         <v>6.0</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="E7" s="6"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="2">
+      <c r="A8" s="3">
         <v>7.0</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="E8" s="6"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="2">
+      <c r="A9" s="3">
         <v>8.0</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="E9" s="6"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="2">
+      <c r="A10" s="3">
         <v>9.0</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="2">
+      <c r="A11" s="3">
         <v>10.0</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="E11" s="6"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="2">
+      <c r="A12" s="3">
         <v>11.0</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="E12" s="6"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="2">
+      <c r="A13" s="3">
         <v>12.0</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="E13" s="6"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="2">
+      <c r="A14" s="3">
         <v>13.0</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="E14" s="6"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="2">
+      <c r="A15" s="3">
         <v>14.0</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="E15" s="6"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="2">
+      <c r="A16" s="3">
         <v>15.0</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="E16" s="6"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="2">
+      <c r="A17" s="3">
         <v>16.0</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="E17" s="6"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="2">
+      <c r="A18" s="3">
         <v>17.0</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="E18" s="6"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="2">
+      <c r="A19" s="3">
         <v>18.0</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="E19" s="6"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="2">
+      <c r="A20" s="3">
         <v>19.0</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="E20" s="6"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="2">
+      <c r="A21" s="3">
         <v>20.0</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="E21" s="6"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="2">
+      <c r="A22" s="3">
         <v>21.0</v>
       </c>
-      <c r="B22" s="6"/>
-      <c r="E22" s="6"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="2">
+      <c r="A23" s="3">
         <v>22.0</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="E23" s="6"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="2">
+      <c r="A24" s="3">
         <v>23.0</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="E24" s="6"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="2">
+      <c r="A25" s="3">
         <v>24.0</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="E25" s="6"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="2">
+      <c r="A26" s="3">
         <v>25.0</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="E26" s="6"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="2">
+      <c r="A27" s="3">
         <v>26.0</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="E27" s="6"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="2">
+      <c r="A28" s="3">
         <v>27.0</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="E28" s="6"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="2">
+      <c r="A29" s="3">
         <v>28.0</v>
       </c>
-      <c r="B29" s="6"/>
-      <c r="E29" s="6"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="2">
+      <c r="A30" s="3">
         <v>29.0</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="E30" s="6"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="2">
+      <c r="A31" s="3">
         <v>30.0</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="E31" s="6"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="B32" s="7"/>
-      <c r="E32" s="7"/>
+      <c r="B32" s="8"/>
+      <c r="E32" s="8"/>
     </row>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
@@ -1643,14 +1726,15 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId2" ref="E2"/>
+    <hyperlink r:id="rId3" ref="E3"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId3"/>
-  <legacyDrawing r:id="rId4"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
   <tableParts count="1">
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>